<commit_message>
cambios en reportes aplicacion
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyeto/Evidencias de Sistema/Aplicación/exel para llenar tablas/TablaServicios.xlsx
+++ b/Fase 2/Evidencias Proyeto/Evidencias de Sistema/Aplicación/exel para llenar tablas/TablaServicios.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matia\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matia\Desktop\Capstone\ProyectoTransporte\Fase 2\Evidencias Proyeto\Evidencias de Sistema\Aplicación\exel para llenar tablas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D89EA22-7D9F-467D-AD51-AC911F3BDA59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C28992-B36D-4D39-A7DF-E8D9CFD0DDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{957EC373-37DC-4A66-8AE7-EF817FFC2B60}"/>
+    <workbookView xWindow="-27705" yWindow="2340" windowWidth="24075" windowHeight="12570" xr2:uid="{957EC373-37DC-4A66-8AE7-EF817FFC2B60}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -183,7 +183,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -527,12 +527,14 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="35.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
     <col min="6" max="6" width="15.140625" customWidth="1"/>
     <col min="7" max="7" width="19.140625" customWidth="1"/>
+    <col min="8" max="8" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>